<commit_message>
price_bank: sheet title category over sheet abbreviation, indexed merges, more real-structure fixtures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UK2gboVRJ1TbJ9N2kjdotp
</commit_message>
<xml_diff>
--- a/price_bank/test/fixtures/PEP-Rev.140205_Sample_4.xlsx
+++ b/price_bank/test/fixtures/PEP-Rev.140205_Sample_4.xlsx
@@ -16,9 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P.EL" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P.IN" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P.PI" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P.LAB" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C.mECHANICAL" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E.Mechanic" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P.PL" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P.LAB" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C.mECHANICAL" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E.Mechanic" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -648,6 +649,438 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ITEM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>DESCRIPTION</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>QUANTITY</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>MATERIAL</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>هزینه واحد خرید بدون ضریب</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>هزینه کل بدون ضریب</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>خرید</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> ترخیص</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حمل </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PIPELINE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SIZE(in)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LENGTH(M)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Euro</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Euro</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Rls</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Rls</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> احداث خط لوله انتقال نفت نمکی  از واحد بهره برداری نمونه 4 به واحد نمک زدایی نمونه  4 ب</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>20"</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>400</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API 5L GR.X52/SCH.30/NACE </t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>300.7517562690128</v>
+      </c>
+      <c r="H4" t="n">
+        <v>116808</v>
+      </c>
+      <c r="I4" t="n">
+        <v>16513703443</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2204077501</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> احداث خط لوله انتقال نفت نمک زدایی شده 20 اینچ روزمینی با جنس API 5L GR.X52/SCH.30/NACE   از واحد نمک زدایی نمونه 4 به واحد بهره برداری نمونه 4 به طول تقریبی 1500 متر.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>20"</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>400</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API 5L GR.X52/SCH.30/NACE </t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>300.7517562690128</v>
+      </c>
+      <c r="H5" t="n">
+        <v>116808</v>
+      </c>
+      <c r="I5" t="n">
+        <v>16513703443</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2204077501</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ساپورت فلزی و فونداسیون (بر اساس تناژ)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>C.S.</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>1127054396</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تعویض خط لوله انتقال نفت از واحد بهره برداری پازنان 2 به واحد بهره برداری نمونه 2  با سایز 12 اینچ  </t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12"</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>19647</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>API 5L GR.X52/SCH.40</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>211.8932828258954</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3531709</v>
+      </c>
+      <c r="I7" t="n">
+        <v>210058885830</v>
+      </c>
+      <c r="J7" t="n">
+        <v>20598883111</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ساپورت فلزی و فونداسیون(61000/کیلو)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2661726699</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>جابجایی خط فشار بالای گاز موجود در سمت شرق سایت و احداث مجدد آن در فاصله  حداقل 200 متر از حصار تسهیلات بیرون واحد</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4"</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>API5L GR.X52/SCH.80/NACE</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>31.4422290644877</v>
+      </c>
+      <c r="H9" t="n">
+        <v>66950</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3340545781</v>
+      </c>
+      <c r="J9" t="n">
+        <v>666301589</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">احداث خط لوله انتقال گاز 6 اینچ فلزی با جنس API5L GR.X52/SCH.80/NACE به صورت روزمینی از واحد بهره برداری نمونه 4 به واحد نمک زدایی نمونه 4 </t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>6"</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>500</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>API5L GR.X52/SCH.80/NACE</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>71.08677875449393</v>
+      </c>
+      <c r="H10" t="n">
+        <v>47765</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2444473200</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1256522295</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>·احداث خط انتقال آب 6 اینچ فلزی با جنس API 5L0 به صورت رو زمینی  از تصفیه خانه خیر آباد  به واحدنمکزدایی نمونه-4</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6"</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>API 5L GR.X52/SCH.STD</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>71.08677875449393</v>
+      </c>
+      <c r="H11" t="n">
+        <v>109686</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5908771681</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2204077501</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  احداث  خط لوله انتقال آب ازاد  غیر فلزی با جنس RTP  زیر زمینی از واحد بهره برداری نمونه-4 به واحدنمکزدایی نمونه-4</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>4"</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>500</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>RTP</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>133.9712368834693</v>
+      </c>
+      <c r="H12" t="n">
+        <v>41446</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4986320488</v>
+      </c>
+      <c r="J12" t="n">
+        <v>879127129</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="F1:F3"/>
+    <mergeCell ref="D1:E2"/>
+    <mergeCell ref="B1:C2"/>
+    <mergeCell ref="G1:G2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -946,7 +1379,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1744,7 +2177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>